<commit_message>
ajustado a criação do exe
</commit_message>
<xml_diff>
--- a/template/FT.xlsx
+++ b/template/FT.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="52">
   <si>
     <t>FICHA DE TEMPO</t>
   </si>
@@ -213,12 +213,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Deslocamento Juiz de Fora - MG  para Araraquara - SP</t>
-  </si>
-  <si>
-    <t>PRÉ - TAF PSU, Ponto a Ponto do painel ensaios elétricos do painel.</t>
   </si>
   <si>
     <t>MEGAWATT SISTEMAS</t>
@@ -1448,164 +1442,6 @@
     <xf numFmtId="168" fontId="10" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="57" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="9" fillId="7" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1674,6 +1510,164 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -11528,7 +11522,7 @@
         <xdr:cNvPr id="2" name="Text Box 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{C4AD235F-88DF-40AC-B289-1354F7BC153A}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C4AD235F-88DF-40AC-B289-1354F7BC153A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -11959,7 +11953,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -11992,63 +11986,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" s="3" customFormat="1" ht="25.2" x14ac:dyDescent="0.25">
-      <c r="A1" s="161" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="162"/>
-      <c r="C1" s="162"/>
-      <c r="D1" s="162"/>
-      <c r="E1" s="162"/>
-      <c r="F1" s="165">
+      <c r="A1" s="114" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="115"/>
+      <c r="C1" s="115"/>
+      <c r="D1" s="115"/>
+      <c r="E1" s="115"/>
+      <c r="F1" s="118">
         <f>A8</f>
         <v>0</v>
       </c>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="167" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="167"/>
-      <c r="K1" s="167"/>
-      <c r="L1" s="167"/>
-      <c r="M1" s="167"/>
-      <c r="N1" s="167"/>
-      <c r="O1" s="167"/>
-      <c r="P1" s="167"/>
-      <c r="Q1" s="167"/>
-      <c r="R1" s="167"/>
-      <c r="S1" s="167"/>
-      <c r="T1" s="167"/>
-      <c r="U1" s="168"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
+      <c r="U1" s="121"/>
       <c r="V1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="W1" s="2"/>
     </row>
     <row r="2" spans="1:32" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A2" s="163"/>
-      <c r="B2" s="164"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="166"/>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
+      <c r="A2" s="116"/>
+      <c r="B2" s="117"/>
+      <c r="C2" s="117"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
       <c r="I2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="169"/>
-      <c r="K2" s="170"/>
-      <c r="L2" s="170"/>
-      <c r="M2" s="170"/>
-      <c r="N2" s="170"/>
-      <c r="O2" s="170"/>
-      <c r="P2" s="170"/>
-      <c r="Q2" s="170"/>
-      <c r="R2" s="170"/>
-      <c r="S2" s="170"/>
-      <c r="T2" s="170"/>
-      <c r="U2" s="171"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="123"/>
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
+      <c r="O2" s="123"/>
+      <c r="P2" s="123"/>
+      <c r="Q2" s="123"/>
+      <c r="R2" s="123"/>
+      <c r="S2" s="123"/>
+      <c r="T2" s="123"/>
+      <c r="U2" s="124"/>
       <c r="V2" s="5" t="s">
         <v>3</v>
       </c>
@@ -12059,25 +12053,25 @@
         <v>4</v>
       </c>
       <c r="B3" s="8"/>
-      <c r="C3" s="172"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="173"/>
-      <c r="F3" s="173"/>
-      <c r="G3" s="173"/>
-      <c r="H3" s="173"/>
-      <c r="I3" s="173"/>
-      <c r="J3" s="173"/>
-      <c r="K3" s="173"/>
-      <c r="L3" s="173"/>
-      <c r="M3" s="174"/>
+      <c r="C3" s="125"/>
+      <c r="D3" s="126"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="126"/>
+      <c r="J3" s="126"/>
+      <c r="K3" s="126"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="127"/>
       <c r="N3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="175"/>
-      <c r="P3" s="176"/>
+      <c r="O3" s="128"/>
+      <c r="P3" s="129"/>
       <c r="Q3" s="9"/>
-      <c r="R3" s="177"/>
-      <c r="S3" s="178"/>
+      <c r="R3" s="130"/>
+      <c r="S3" s="131"/>
       <c r="T3" s="10" t="s">
         <v>6</v>
       </c>
@@ -12092,22 +12086,22 @@
         <v>8</v>
       </c>
       <c r="B4" s="14"/>
-      <c r="C4" s="134"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="135"/>
-      <c r="F4" s="135"/>
-      <c r="G4" s="135"/>
-      <c r="H4" s="135"/>
-      <c r="I4" s="135"/>
-      <c r="J4" s="135"/>
-      <c r="K4" s="135"/>
-      <c r="L4" s="135"/>
-      <c r="M4" s="136"/>
+      <c r="C4" s="150"/>
+      <c r="D4" s="151"/>
+      <c r="E4" s="151"/>
+      <c r="F4" s="151"/>
+      <c r="G4" s="151"/>
+      <c r="H4" s="151"/>
+      <c r="I4" s="151"/>
+      <c r="J4" s="151"/>
+      <c r="K4" s="151"/>
+      <c r="L4" s="151"/>
+      <c r="M4" s="152"/>
       <c r="N4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="134"/>
-      <c r="P4" s="137"/>
+      <c r="O4" s="150"/>
+      <c r="P4" s="153"/>
       <c r="Q4" s="17" t="s">
         <v>10</v>
       </c>
@@ -12126,25 +12120,25 @@
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="22"/>
-      <c r="D5" s="138" t="s">
+      <c r="D5" s="154" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="139"/>
-      <c r="F5" s="140"/>
-      <c r="G5" s="140"/>
-      <c r="H5" s="140"/>
-      <c r="I5" s="140"/>
-      <c r="J5" s="140"/>
-      <c r="K5" s="140"/>
-      <c r="L5" s="140"/>
-      <c r="M5" s="140"/>
-      <c r="N5" s="140"/>
-      <c r="O5" s="140"/>
+      <c r="E5" s="155"/>
+      <c r="F5" s="156"/>
+      <c r="G5" s="156"/>
+      <c r="H5" s="156"/>
+      <c r="I5" s="156"/>
+      <c r="J5" s="156"/>
+      <c r="K5" s="156"/>
+      <c r="L5" s="156"/>
+      <c r="M5" s="156"/>
+      <c r="N5" s="156"/>
+      <c r="O5" s="156"/>
       <c r="P5" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="Q5" s="141"/>
-      <c r="R5" s="142"/>
+      <c r="Q5" s="157"/>
+      <c r="R5" s="158"/>
       <c r="S5" s="25" t="s">
         <v>15</v>
       </c>
@@ -12190,33 +12184,33 @@
       <c r="AF6" s="30"/>
     </row>
     <row r="7" spans="1:32" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="143" t="s">
+      <c r="A7" s="132" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="144"/>
-      <c r="C7" s="145" t="s">
+      <c r="B7" s="133"/>
+      <c r="C7" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="146"/>
-      <c r="E7" s="146"/>
-      <c r="F7" s="146"/>
-      <c r="G7" s="146"/>
-      <c r="H7" s="146"/>
-      <c r="I7" s="146"/>
-      <c r="J7" s="147"/>
-      <c r="K7" s="148" t="s">
+      <c r="D7" s="135"/>
+      <c r="E7" s="135"/>
+      <c r="F7" s="135"/>
+      <c r="G7" s="135"/>
+      <c r="H7" s="135"/>
+      <c r="I7" s="135"/>
+      <c r="J7" s="136"/>
+      <c r="K7" s="137" t="s">
         <v>19</v>
       </c>
-      <c r="L7" s="149"/>
-      <c r="M7" s="149"/>
-      <c r="N7" s="150"/>
-      <c r="O7" s="151" t="s">
+      <c r="L7" s="138"/>
+      <c r="M7" s="138"/>
+      <c r="N7" s="139"/>
+      <c r="O7" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="P7" s="152"/>
-      <c r="Q7" s="152"/>
-      <c r="R7" s="152"/>
-      <c r="S7" s="152"/>
+      <c r="P7" s="141"/>
+      <c r="Q7" s="141"/>
+      <c r="R7" s="141"/>
+      <c r="S7" s="141"/>
       <c r="T7" s="31"/>
       <c r="U7" s="31"/>
       <c r="V7" s="32"/>
@@ -12230,39 +12224,39 @@
       <c r="AF7" s="30"/>
     </row>
     <row r="8" spans="1:32" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="157"/>
-      <c r="B8" s="158"/>
-      <c r="C8" s="127" t="s">
+      <c r="A8" s="146"/>
+      <c r="B8" s="147"/>
+      <c r="C8" s="162" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="128"/>
-      <c r="E8" s="127" t="s">
+      <c r="D8" s="163"/>
+      <c r="E8" s="162" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="128"/>
-      <c r="G8" s="127" t="s">
+      <c r="F8" s="163"/>
+      <c r="G8" s="162" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="128"/>
-      <c r="I8" s="129" t="s">
+      <c r="H8" s="163"/>
+      <c r="I8" s="164" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="128"/>
-      <c r="K8" s="130" t="s">
+      <c r="J8" s="163"/>
+      <c r="K8" s="165" t="s">
         <v>25</v>
       </c>
-      <c r="L8" s="132" t="s">
+      <c r="L8" s="167" t="s">
         <v>26</v>
       </c>
-      <c r="M8" s="133"/>
+      <c r="M8" s="168"/>
       <c r="N8" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="O8" s="153"/>
-      <c r="P8" s="154"/>
-      <c r="Q8" s="154"/>
-      <c r="R8" s="154"/>
-      <c r="S8" s="154"/>
+      <c r="O8" s="142"/>
+      <c r="P8" s="143"/>
+      <c r="Q8" s="143"/>
+      <c r="R8" s="143"/>
+      <c r="S8" s="143"/>
       <c r="T8" s="35"/>
       <c r="U8" s="35"/>
       <c r="V8" s="36"/>
@@ -12276,8 +12270,8 @@
       <c r="AF8" s="30"/>
     </row>
     <row r="9" spans="1:32" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="159"/>
-      <c r="B9" s="160"/>
+      <c r="A9" s="148"/>
+      <c r="B9" s="149"/>
       <c r="C9" s="38" t="s">
         <v>28</v>
       </c>
@@ -12302,7 +12296,7 @@
       <c r="J9" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="131"/>
+      <c r="K9" s="166"/>
       <c r="L9" s="42">
         <v>0.5</v>
       </c>
@@ -12312,11 +12306,11 @@
       <c r="N9" s="44">
         <v>0.3</v>
       </c>
-      <c r="O9" s="155"/>
-      <c r="P9" s="156"/>
-      <c r="Q9" s="156"/>
-      <c r="R9" s="156"/>
-      <c r="S9" s="156"/>
+      <c r="O9" s="144"/>
+      <c r="P9" s="145"/>
+      <c r="Q9" s="145"/>
+      <c r="R9" s="145"/>
+      <c r="S9" s="145"/>
       <c r="T9" s="45"/>
       <c r="U9" s="45"/>
       <c r="V9" s="41"/>
@@ -12372,14 +12366,14 @@
         <f>SUM(AA10,AD10)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="124"/>
-      <c r="P10" s="125"/>
-      <c r="Q10" s="125"/>
-      <c r="R10" s="125"/>
-      <c r="S10" s="125"/>
-      <c r="T10" s="125"/>
-      <c r="U10" s="125"/>
-      <c r="V10" s="126"/>
+      <c r="O10" s="169"/>
+      <c r="P10" s="170"/>
+      <c r="Q10" s="170"/>
+      <c r="R10" s="170"/>
+      <c r="S10" s="170"/>
+      <c r="T10" s="170"/>
+      <c r="U10" s="170"/>
+      <c r="V10" s="171"/>
       <c r="W10" s="59"/>
       <c r="Y10" s="60"/>
       <c r="Z10" s="61"/>
@@ -12435,14 +12429,14 @@
         <f t="shared" ref="N11:N40" si="9">SUM(AA11,AD11)</f>
         <v>0</v>
       </c>
-      <c r="O11" s="121"/>
-      <c r="P11" s="122"/>
-      <c r="Q11" s="122"/>
-      <c r="R11" s="122"/>
-      <c r="S11" s="122"/>
-      <c r="T11" s="122"/>
-      <c r="U11" s="122"/>
-      <c r="V11" s="123"/>
+      <c r="O11" s="159"/>
+      <c r="P11" s="160"/>
+      <c r="Q11" s="160"/>
+      <c r="R11" s="160"/>
+      <c r="S11" s="160"/>
+      <c r="T11" s="160"/>
+      <c r="U11" s="160"/>
+      <c r="V11" s="161"/>
       <c r="W11" s="59"/>
       <c r="Y11" s="60"/>
       <c r="Z11" s="61"/>
@@ -12498,14 +12492,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O12" s="121"/>
-      <c r="P12" s="122"/>
-      <c r="Q12" s="122"/>
-      <c r="R12" s="122"/>
-      <c r="S12" s="122"/>
-      <c r="T12" s="122"/>
-      <c r="U12" s="122"/>
-      <c r="V12" s="123"/>
+      <c r="O12" s="159"/>
+      <c r="P12" s="160"/>
+      <c r="Q12" s="160"/>
+      <c r="R12" s="160"/>
+      <c r="S12" s="160"/>
+      <c r="T12" s="160"/>
+      <c r="U12" s="160"/>
+      <c r="V12" s="161"/>
       <c r="W12" s="59"/>
       <c r="Y12" s="60"/>
       <c r="Z12" s="61"/>
@@ -12561,14 +12555,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O13" s="121"/>
-      <c r="P13" s="122"/>
-      <c r="Q13" s="122"/>
-      <c r="R13" s="122"/>
-      <c r="S13" s="122"/>
-      <c r="T13" s="122"/>
-      <c r="U13" s="122"/>
-      <c r="V13" s="123"/>
+      <c r="O13" s="159"/>
+      <c r="P13" s="160"/>
+      <c r="Q13" s="160"/>
+      <c r="R13" s="160"/>
+      <c r="S13" s="160"/>
+      <c r="T13" s="160"/>
+      <c r="U13" s="160"/>
+      <c r="V13" s="161"/>
       <c r="W13" s="59"/>
       <c r="Y13" s="60"/>
       <c r="Z13" s="61"/>
@@ -12624,14 +12618,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O14" s="121"/>
-      <c r="P14" s="122"/>
-      <c r="Q14" s="122"/>
-      <c r="R14" s="122"/>
-      <c r="S14" s="122"/>
-      <c r="T14" s="122"/>
-      <c r="U14" s="122"/>
-      <c r="V14" s="123"/>
+      <c r="O14" s="159"/>
+      <c r="P14" s="160"/>
+      <c r="Q14" s="160"/>
+      <c r="R14" s="160"/>
+      <c r="S14" s="160"/>
+      <c r="T14" s="160"/>
+      <c r="U14" s="160"/>
+      <c r="V14" s="161"/>
       <c r="W14" s="59"/>
       <c r="Y14" s="60"/>
       <c r="Z14" s="61"/>
@@ -12687,14 +12681,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O15" s="121"/>
-      <c r="P15" s="122"/>
-      <c r="Q15" s="122"/>
-      <c r="R15" s="122"/>
-      <c r="S15" s="122"/>
-      <c r="T15" s="122"/>
-      <c r="U15" s="122"/>
-      <c r="V15" s="123"/>
+      <c r="O15" s="159"/>
+      <c r="P15" s="160"/>
+      <c r="Q15" s="160"/>
+      <c r="R15" s="160"/>
+      <c r="S15" s="160"/>
+      <c r="T15" s="160"/>
+      <c r="U15" s="160"/>
+      <c r="V15" s="161"/>
       <c r="W15" s="59"/>
       <c r="Y15" s="60"/>
       <c r="Z15" s="61"/>
@@ -12750,14 +12744,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O16" s="121"/>
-      <c r="P16" s="122"/>
-      <c r="Q16" s="122"/>
-      <c r="R16" s="122"/>
-      <c r="S16" s="122"/>
-      <c r="T16" s="122"/>
-      <c r="U16" s="122"/>
-      <c r="V16" s="123"/>
+      <c r="O16" s="159"/>
+      <c r="P16" s="160"/>
+      <c r="Q16" s="160"/>
+      <c r="R16" s="160"/>
+      <c r="S16" s="160"/>
+      <c r="T16" s="160"/>
+      <c r="U16" s="160"/>
+      <c r="V16" s="161"/>
       <c r="W16" s="59"/>
       <c r="Y16" s="60"/>
       <c r="Z16" s="61"/>
@@ -12813,14 +12807,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O17" s="121"/>
-      <c r="P17" s="122"/>
-      <c r="Q17" s="122"/>
-      <c r="R17" s="122"/>
-      <c r="S17" s="122"/>
-      <c r="T17" s="122"/>
-      <c r="U17" s="122"/>
-      <c r="V17" s="123"/>
+      <c r="O17" s="159"/>
+      <c r="P17" s="160"/>
+      <c r="Q17" s="160"/>
+      <c r="R17" s="160"/>
+      <c r="S17" s="160"/>
+      <c r="T17" s="160"/>
+      <c r="U17" s="160"/>
+      <c r="V17" s="161"/>
       <c r="W17" s="59"/>
       <c r="Y17" s="60"/>
       <c r="Z17" s="61"/>
@@ -12876,14 +12870,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O18" s="121"/>
-      <c r="P18" s="122"/>
-      <c r="Q18" s="122"/>
-      <c r="R18" s="122"/>
-      <c r="S18" s="122"/>
-      <c r="T18" s="122"/>
-      <c r="U18" s="122"/>
-      <c r="V18" s="123"/>
+      <c r="O18" s="159"/>
+      <c r="P18" s="160"/>
+      <c r="Q18" s="160"/>
+      <c r="R18" s="160"/>
+      <c r="S18" s="160"/>
+      <c r="T18" s="160"/>
+      <c r="U18" s="160"/>
+      <c r="V18" s="161"/>
       <c r="W18" s="59"/>
       <c r="Y18" s="60"/>
       <c r="Z18" s="61"/>
@@ -12939,14 +12933,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O19" s="121"/>
-      <c r="P19" s="122"/>
-      <c r="Q19" s="122"/>
-      <c r="R19" s="122"/>
-      <c r="S19" s="122"/>
-      <c r="T19" s="122"/>
-      <c r="U19" s="122"/>
-      <c r="V19" s="123"/>
+      <c r="O19" s="159"/>
+      <c r="P19" s="160"/>
+      <c r="Q19" s="160"/>
+      <c r="R19" s="160"/>
+      <c r="S19" s="160"/>
+      <c r="T19" s="160"/>
+      <c r="U19" s="160"/>
+      <c r="V19" s="161"/>
       <c r="W19" s="59"/>
       <c r="Y19" s="60"/>
       <c r="Z19" s="61"/>
@@ -13002,14 +12996,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O20" s="121"/>
-      <c r="P20" s="122"/>
-      <c r="Q20" s="122"/>
-      <c r="R20" s="122"/>
-      <c r="S20" s="122"/>
-      <c r="T20" s="122"/>
-      <c r="U20" s="122"/>
-      <c r="V20" s="123"/>
+      <c r="O20" s="159"/>
+      <c r="P20" s="160"/>
+      <c r="Q20" s="160"/>
+      <c r="R20" s="160"/>
+      <c r="S20" s="160"/>
+      <c r="T20" s="160"/>
+      <c r="U20" s="160"/>
+      <c r="V20" s="161"/>
       <c r="W20" s="59"/>
       <c r="Y20" s="60"/>
       <c r="Z20" s="61"/>
@@ -13066,14 +13060,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O21" s="121"/>
-      <c r="P21" s="122"/>
-      <c r="Q21" s="122"/>
-      <c r="R21" s="122"/>
-      <c r="S21" s="122"/>
-      <c r="T21" s="122"/>
-      <c r="U21" s="122"/>
-      <c r="V21" s="123"/>
+      <c r="O21" s="159"/>
+      <c r="P21" s="160"/>
+      <c r="Q21" s="160"/>
+      <c r="R21" s="160"/>
+      <c r="S21" s="160"/>
+      <c r="T21" s="160"/>
+      <c r="U21" s="160"/>
+      <c r="V21" s="161"/>
       <c r="W21" s="59"/>
       <c r="Y21" s="60"/>
       <c r="Z21" s="61"/>
@@ -13130,14 +13124,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O22" s="121"/>
-      <c r="P22" s="122"/>
-      <c r="Q22" s="122"/>
-      <c r="R22" s="122"/>
-      <c r="S22" s="122"/>
-      <c r="T22" s="122"/>
-      <c r="U22" s="122"/>
-      <c r="V22" s="123"/>
+      <c r="O22" s="159"/>
+      <c r="P22" s="160"/>
+      <c r="Q22" s="160"/>
+      <c r="R22" s="160"/>
+      <c r="S22" s="160"/>
+      <c r="T22" s="160"/>
+      <c r="U22" s="160"/>
+      <c r="V22" s="161"/>
       <c r="W22" s="59"/>
       <c r="Y22" s="60"/>
       <c r="Z22" s="61"/>
@@ -13193,14 +13187,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O23" s="121"/>
-      <c r="P23" s="122"/>
-      <c r="Q23" s="122"/>
-      <c r="R23" s="122"/>
-      <c r="S23" s="122"/>
-      <c r="T23" s="122"/>
-      <c r="U23" s="122"/>
-      <c r="V23" s="123"/>
+      <c r="O23" s="159"/>
+      <c r="P23" s="160"/>
+      <c r="Q23" s="160"/>
+      <c r="R23" s="160"/>
+      <c r="S23" s="160"/>
+      <c r="T23" s="160"/>
+      <c r="U23" s="160"/>
+      <c r="V23" s="161"/>
       <c r="W23" s="59"/>
       <c r="Y23" s="60"/>
       <c r="Z23" s="61"/>
@@ -13256,14 +13250,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O24" s="121"/>
-      <c r="P24" s="122"/>
-      <c r="Q24" s="122"/>
-      <c r="R24" s="122"/>
-      <c r="S24" s="122"/>
-      <c r="T24" s="122"/>
-      <c r="U24" s="122"/>
-      <c r="V24" s="123"/>
+      <c r="O24" s="159"/>
+      <c r="P24" s="160"/>
+      <c r="Q24" s="160"/>
+      <c r="R24" s="160"/>
+      <c r="S24" s="160"/>
+      <c r="T24" s="160"/>
+      <c r="U24" s="160"/>
+      <c r="V24" s="161"/>
       <c r="W24" s="59"/>
       <c r="Y24" s="60"/>
       <c r="Z24" s="61"/>
@@ -13321,14 +13315,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O25" s="121"/>
-      <c r="P25" s="122"/>
-      <c r="Q25" s="122"/>
-      <c r="R25" s="122"/>
-      <c r="S25" s="122"/>
-      <c r="T25" s="122"/>
-      <c r="U25" s="122"/>
-      <c r="V25" s="123"/>
+      <c r="O25" s="159"/>
+      <c r="P25" s="160"/>
+      <c r="Q25" s="160"/>
+      <c r="R25" s="160"/>
+      <c r="S25" s="160"/>
+      <c r="T25" s="160"/>
+      <c r="U25" s="160"/>
+      <c r="V25" s="161"/>
       <c r="W25" s="59"/>
       <c r="Y25" s="60"/>
       <c r="Z25" s="61"/>
@@ -13384,14 +13378,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O26" s="121"/>
-      <c r="P26" s="122"/>
-      <c r="Q26" s="122"/>
-      <c r="R26" s="122"/>
-      <c r="S26" s="122"/>
-      <c r="T26" s="122"/>
-      <c r="U26" s="122"/>
-      <c r="V26" s="123"/>
+      <c r="O26" s="159"/>
+      <c r="P26" s="160"/>
+      <c r="Q26" s="160"/>
+      <c r="R26" s="160"/>
+      <c r="S26" s="160"/>
+      <c r="T26" s="160"/>
+      <c r="U26" s="160"/>
+      <c r="V26" s="161"/>
       <c r="W26" s="59"/>
       <c r="Y26" s="60"/>
       <c r="Z26" s="61"/>
@@ -13447,14 +13441,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O27" s="121"/>
-      <c r="P27" s="122"/>
-      <c r="Q27" s="122"/>
-      <c r="R27" s="122"/>
-      <c r="S27" s="122"/>
-      <c r="T27" s="122"/>
-      <c r="U27" s="122"/>
-      <c r="V27" s="123"/>
+      <c r="O27" s="159"/>
+      <c r="P27" s="160"/>
+      <c r="Q27" s="160"/>
+      <c r="R27" s="160"/>
+      <c r="S27" s="160"/>
+      <c r="T27" s="160"/>
+      <c r="U27" s="160"/>
+      <c r="V27" s="161"/>
       <c r="W27" s="59"/>
       <c r="Y27" s="60"/>
       <c r="Z27" s="61"/>
@@ -13510,14 +13504,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O28" s="121"/>
-      <c r="P28" s="122"/>
-      <c r="Q28" s="122"/>
-      <c r="R28" s="122"/>
-      <c r="S28" s="122"/>
-      <c r="T28" s="122"/>
-      <c r="U28" s="122"/>
-      <c r="V28" s="123"/>
+      <c r="O28" s="159"/>
+      <c r="P28" s="160"/>
+      <c r="Q28" s="160"/>
+      <c r="R28" s="160"/>
+      <c r="S28" s="160"/>
+      <c r="T28" s="160"/>
+      <c r="U28" s="160"/>
+      <c r="V28" s="161"/>
       <c r="W28" s="59"/>
       <c r="Y28" s="60"/>
       <c r="Z28" s="61"/>
@@ -13573,14 +13567,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O29" s="121"/>
-      <c r="P29" s="122"/>
-      <c r="Q29" s="122"/>
-      <c r="R29" s="122"/>
-      <c r="S29" s="122"/>
-      <c r="T29" s="122"/>
-      <c r="U29" s="122"/>
-      <c r="V29" s="123"/>
+      <c r="O29" s="159"/>
+      <c r="P29" s="160"/>
+      <c r="Q29" s="160"/>
+      <c r="R29" s="160"/>
+      <c r="S29" s="160"/>
+      <c r="T29" s="160"/>
+      <c r="U29" s="160"/>
+      <c r="V29" s="161"/>
       <c r="W29" s="59"/>
       <c r="Y29" s="60"/>
       <c r="Z29" s="61"/>
@@ -13638,14 +13632,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O30" s="121"/>
-      <c r="P30" s="122"/>
-      <c r="Q30" s="122"/>
-      <c r="R30" s="122"/>
-      <c r="S30" s="122"/>
-      <c r="T30" s="122"/>
-      <c r="U30" s="122"/>
-      <c r="V30" s="123"/>
+      <c r="O30" s="159"/>
+      <c r="P30" s="160"/>
+      <c r="Q30" s="160"/>
+      <c r="R30" s="160"/>
+      <c r="S30" s="160"/>
+      <c r="T30" s="160"/>
+      <c r="U30" s="160"/>
+      <c r="V30" s="161"/>
       <c r="W30" s="70"/>
       <c r="Y30" s="72"/>
       <c r="Z30" s="73"/>
@@ -13701,14 +13695,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O31" s="121"/>
-      <c r="P31" s="122"/>
-      <c r="Q31" s="122"/>
-      <c r="R31" s="122"/>
-      <c r="S31" s="122"/>
-      <c r="T31" s="122"/>
-      <c r="U31" s="122"/>
-      <c r="V31" s="123"/>
+      <c r="O31" s="159"/>
+      <c r="P31" s="160"/>
+      <c r="Q31" s="160"/>
+      <c r="R31" s="160"/>
+      <c r="S31" s="160"/>
+      <c r="T31" s="160"/>
+      <c r="U31" s="160"/>
+      <c r="V31" s="161"/>
       <c r="W31" s="70"/>
       <c r="Y31" s="72"/>
       <c r="Z31" s="73"/>
@@ -13764,14 +13758,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O32" s="121"/>
-      <c r="P32" s="122"/>
-      <c r="Q32" s="122"/>
-      <c r="R32" s="122"/>
-      <c r="S32" s="122"/>
-      <c r="T32" s="122"/>
-      <c r="U32" s="122"/>
-      <c r="V32" s="123"/>
+      <c r="O32" s="159"/>
+      <c r="P32" s="160"/>
+      <c r="Q32" s="160"/>
+      <c r="R32" s="160"/>
+      <c r="S32" s="160"/>
+      <c r="T32" s="160"/>
+      <c r="U32" s="160"/>
+      <c r="V32" s="161"/>
       <c r="W32" s="59"/>
       <c r="Y32" s="60"/>
       <c r="Z32" s="61"/>
@@ -13827,14 +13821,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O33" s="121"/>
-      <c r="P33" s="122"/>
-      <c r="Q33" s="122"/>
-      <c r="R33" s="122"/>
-      <c r="S33" s="122"/>
-      <c r="T33" s="122"/>
-      <c r="U33" s="122"/>
-      <c r="V33" s="123"/>
+      <c r="O33" s="159"/>
+      <c r="P33" s="160"/>
+      <c r="Q33" s="160"/>
+      <c r="R33" s="160"/>
+      <c r="S33" s="160"/>
+      <c r="T33" s="160"/>
+      <c r="U33" s="160"/>
+      <c r="V33" s="161"/>
       <c r="W33" s="59"/>
       <c r="Y33" s="60"/>
       <c r="Z33" s="61"/>
@@ -13890,14 +13884,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O34" s="121"/>
-      <c r="P34" s="122"/>
-      <c r="Q34" s="122"/>
-      <c r="R34" s="122"/>
-      <c r="S34" s="122"/>
-      <c r="T34" s="122"/>
-      <c r="U34" s="122"/>
-      <c r="V34" s="123"/>
+      <c r="O34" s="159"/>
+      <c r="P34" s="160"/>
+      <c r="Q34" s="160"/>
+      <c r="R34" s="160"/>
+      <c r="S34" s="160"/>
+      <c r="T34" s="160"/>
+      <c r="U34" s="160"/>
+      <c r="V34" s="161"/>
       <c r="W34" s="59"/>
       <c r="Y34" s="60"/>
       <c r="Z34" s="60"/>
@@ -13951,14 +13945,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O35" s="121"/>
-      <c r="P35" s="122"/>
-      <c r="Q35" s="122"/>
-      <c r="R35" s="122"/>
-      <c r="S35" s="122"/>
-      <c r="T35" s="122"/>
-      <c r="U35" s="122"/>
-      <c r="V35" s="123"/>
+      <c r="O35" s="159"/>
+      <c r="P35" s="160"/>
+      <c r="Q35" s="160"/>
+      <c r="R35" s="160"/>
+      <c r="S35" s="160"/>
+      <c r="T35" s="160"/>
+      <c r="U35" s="160"/>
+      <c r="V35" s="161"/>
       <c r="W35" s="59"/>
       <c r="Y35" s="60"/>
       <c r="Z35" s="60"/>
@@ -14012,14 +14006,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O36" s="121"/>
-      <c r="P36" s="122"/>
-      <c r="Q36" s="122"/>
-      <c r="R36" s="122"/>
-      <c r="S36" s="122"/>
-      <c r="T36" s="122"/>
-      <c r="U36" s="122"/>
-      <c r="V36" s="123"/>
+      <c r="O36" s="159"/>
+      <c r="P36" s="160"/>
+      <c r="Q36" s="160"/>
+      <c r="R36" s="160"/>
+      <c r="S36" s="160"/>
+      <c r="T36" s="160"/>
+      <c r="U36" s="160"/>
+      <c r="V36" s="161"/>
       <c r="W36" s="59"/>
       <c r="Y36" s="60"/>
       <c r="Z36" s="60"/>
@@ -14073,14 +14067,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O37" s="121"/>
-      <c r="P37" s="122"/>
-      <c r="Q37" s="122"/>
-      <c r="R37" s="122"/>
-      <c r="S37" s="122"/>
-      <c r="T37" s="122"/>
-      <c r="U37" s="122"/>
-      <c r="V37" s="123"/>
+      <c r="O37" s="159"/>
+      <c r="P37" s="160"/>
+      <c r="Q37" s="160"/>
+      <c r="R37" s="160"/>
+      <c r="S37" s="160"/>
+      <c r="T37" s="160"/>
+      <c r="U37" s="160"/>
+      <c r="V37" s="161"/>
       <c r="W37" s="59"/>
       <c r="Y37" s="60"/>
       <c r="Z37" s="60"/>
@@ -14134,14 +14128,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O38" s="121"/>
-      <c r="P38" s="122"/>
-      <c r="Q38" s="122"/>
-      <c r="R38" s="122"/>
-      <c r="S38" s="122"/>
-      <c r="T38" s="122"/>
-      <c r="U38" s="122"/>
-      <c r="V38" s="123"/>
+      <c r="O38" s="159"/>
+      <c r="P38" s="160"/>
+      <c r="Q38" s="160"/>
+      <c r="R38" s="160"/>
+      <c r="S38" s="160"/>
+      <c r="T38" s="160"/>
+      <c r="U38" s="160"/>
+      <c r="V38" s="161"/>
       <c r="W38" s="59"/>
       <c r="Y38" s="60"/>
       <c r="Z38" s="60"/>
@@ -14195,16 +14189,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O39" s="121" t="s">
-        <v>51</v>
-      </c>
-      <c r="P39" s="122"/>
-      <c r="Q39" s="122"/>
-      <c r="R39" s="122"/>
-      <c r="S39" s="122"/>
-      <c r="T39" s="122"/>
-      <c r="U39" s="122"/>
-      <c r="V39" s="123"/>
+      <c r="O39" s="159"/>
+      <c r="P39" s="160"/>
+      <c r="Q39" s="160"/>
+      <c r="R39" s="160"/>
+      <c r="S39" s="160"/>
+      <c r="T39" s="160"/>
+      <c r="U39" s="160"/>
+      <c r="V39" s="161"/>
       <c r="W39" s="59"/>
       <c r="Y39" s="60"/>
       <c r="Z39" s="60"/>
@@ -14258,16 +14250,14 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="O40" s="124" t="s">
-        <v>52</v>
-      </c>
-      <c r="P40" s="125"/>
-      <c r="Q40" s="125"/>
-      <c r="R40" s="125"/>
-      <c r="S40" s="125"/>
-      <c r="T40" s="125"/>
-      <c r="U40" s="125"/>
-      <c r="V40" s="126"/>
+      <c r="O40" s="169"/>
+      <c r="P40" s="170"/>
+      <c r="Q40" s="170"/>
+      <c r="R40" s="170"/>
+      <c r="S40" s="170"/>
+      <c r="T40" s="170"/>
+      <c r="U40" s="170"/>
+      <c r="V40" s="171"/>
       <c r="W40" s="81"/>
       <c r="Y40" s="60"/>
       <c r="Z40" s="60"/>
@@ -14289,18 +14279,18 @@
       </c>
     </row>
     <row r="41" spans="1:32" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="117" t="s">
+      <c r="A41" s="172" t="s">
         <v>35</v>
       </c>
-      <c r="B41" s="118"/>
-      <c r="C41" s="119"/>
-      <c r="D41" s="119"/>
-      <c r="E41" s="119"/>
-      <c r="F41" s="119"/>
-      <c r="G41" s="119"/>
-      <c r="H41" s="119"/>
-      <c r="I41" s="119"/>
-      <c r="J41" s="120"/>
+      <c r="B41" s="173"/>
+      <c r="C41" s="174"/>
+      <c r="D41" s="174"/>
+      <c r="E41" s="174"/>
+      <c r="F41" s="174"/>
+      <c r="G41" s="174"/>
+      <c r="H41" s="174"/>
+      <c r="I41" s="174"/>
+      <c r="J41" s="175"/>
       <c r="K41" s="83">
         <f>SUM(K10:K40)</f>
         <v>0</v>
@@ -14382,28 +14372,28 @@
       <c r="W43" s="28"/>
     </row>
     <row r="44" spans="1:32" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="114" t="s">
+      <c r="A44" s="176" t="s">
         <v>36</v>
       </c>
-      <c r="B44" s="115"/>
-      <c r="C44" s="115"/>
-      <c r="D44" s="115"/>
-      <c r="E44" s="116"/>
-      <c r="F44" s="114" t="s">
+      <c r="B44" s="177"/>
+      <c r="C44" s="177"/>
+      <c r="D44" s="177"/>
+      <c r="E44" s="178"/>
+      <c r="F44" s="176" t="s">
         <v>37</v>
       </c>
-      <c r="G44" s="115"/>
-      <c r="H44" s="115"/>
-      <c r="I44" s="115"/>
-      <c r="J44" s="115"/>
-      <c r="K44" s="116"/>
+      <c r="G44" s="177"/>
+      <c r="H44" s="177"/>
+      <c r="I44" s="177"/>
+      <c r="J44" s="177"/>
+      <c r="K44" s="178"/>
       <c r="L44" s="91"/>
-      <c r="M44" s="115"/>
-      <c r="N44" s="115"/>
-      <c r="O44" s="115"/>
-      <c r="P44" s="115"/>
-      <c r="Q44" s="115"/>
-      <c r="R44" s="116"/>
+      <c r="M44" s="177"/>
+      <c r="N44" s="177"/>
+      <c r="O44" s="177"/>
+      <c r="P44" s="177"/>
+      <c r="Q44" s="177"/>
+      <c r="R44" s="178"/>
       <c r="S44" s="92" t="s">
         <v>38</v>
       </c>
@@ -14453,28 +14443,28 @@
       <c r="W48" s="96"/>
     </row>
     <row r="49" spans="1:23" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="114" t="s">
+      <c r="A49" s="176" t="s">
         <v>41</v>
       </c>
-      <c r="B49" s="115"/>
-      <c r="C49" s="115"/>
-      <c r="D49" s="115"/>
-      <c r="E49" s="116"/>
-      <c r="F49" s="114" t="s">
+      <c r="B49" s="177"/>
+      <c r="C49" s="177"/>
+      <c r="D49" s="177"/>
+      <c r="E49" s="178"/>
+      <c r="F49" s="176" t="s">
         <v>41</v>
       </c>
-      <c r="G49" s="115"/>
-      <c r="H49" s="115"/>
-      <c r="I49" s="115"/>
-      <c r="J49" s="115"/>
-      <c r="K49" s="116"/>
+      <c r="G49" s="177"/>
+      <c r="H49" s="177"/>
+      <c r="I49" s="177"/>
+      <c r="J49" s="177"/>
+      <c r="K49" s="178"/>
       <c r="L49" s="91"/>
-      <c r="M49" s="115"/>
-      <c r="N49" s="115"/>
-      <c r="O49" s="115"/>
-      <c r="P49" s="115"/>
-      <c r="Q49" s="115"/>
-      <c r="R49" s="116"/>
+      <c r="M49" s="177"/>
+      <c r="N49" s="177"/>
+      <c r="O49" s="177"/>
+      <c r="P49" s="177"/>
+      <c r="Q49" s="177"/>
+      <c r="R49" s="178"/>
       <c r="S49" s="98" t="s">
         <v>42</v>
       </c>
@@ -14507,23 +14497,38 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="LGR5A+3MPBKt5QBDWiYbbiOZZmozoQgK7sbVuTyepsXrIjpIlZuJHyAYOaJk2Y3LyXlZFyNKGAgumbfYJCaXEQ==" saltValue="GcsowBuP4E/OC1BprCxdwQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="63">
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="F1:H2"/>
-    <mergeCell ref="I1:U1"/>
-    <mergeCell ref="J2:U2"/>
-    <mergeCell ref="C3:M3"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="O7:S9"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C4:M4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:O5"/>
-    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="F44:K44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="O44:R44"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="F49:K49"/>
+    <mergeCell ref="M49:N49"/>
+    <mergeCell ref="O49:R49"/>
+    <mergeCell ref="A41:J41"/>
+    <mergeCell ref="O30:V30"/>
+    <mergeCell ref="O31:V31"/>
+    <mergeCell ref="O32:V32"/>
+    <mergeCell ref="O33:V33"/>
+    <mergeCell ref="O34:V34"/>
+    <mergeCell ref="O35:V35"/>
+    <mergeCell ref="O36:V36"/>
+    <mergeCell ref="O37:V37"/>
+    <mergeCell ref="O38:V38"/>
+    <mergeCell ref="O39:V39"/>
+    <mergeCell ref="O40:V40"/>
+    <mergeCell ref="O29:V29"/>
+    <mergeCell ref="O18:V18"/>
+    <mergeCell ref="O19:V19"/>
+    <mergeCell ref="O20:V20"/>
+    <mergeCell ref="O21:V21"/>
+    <mergeCell ref="O22:V22"/>
+    <mergeCell ref="O23:V23"/>
+    <mergeCell ref="O24:V24"/>
+    <mergeCell ref="O25:V25"/>
+    <mergeCell ref="O26:V26"/>
+    <mergeCell ref="O27:V27"/>
+    <mergeCell ref="O28:V28"/>
     <mergeCell ref="O17:V17"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
@@ -14538,38 +14543,23 @@
     <mergeCell ref="O16:V16"/>
     <mergeCell ref="O11:V11"/>
     <mergeCell ref="O12:V12"/>
-    <mergeCell ref="O29:V29"/>
-    <mergeCell ref="O18:V18"/>
-    <mergeCell ref="O19:V19"/>
-    <mergeCell ref="O20:V20"/>
-    <mergeCell ref="O21:V21"/>
-    <mergeCell ref="O22:V22"/>
-    <mergeCell ref="O23:V23"/>
-    <mergeCell ref="O24:V24"/>
-    <mergeCell ref="O25:V25"/>
-    <mergeCell ref="O26:V26"/>
-    <mergeCell ref="O27:V27"/>
-    <mergeCell ref="O28:V28"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="O30:V30"/>
-    <mergeCell ref="O31:V31"/>
-    <mergeCell ref="O32:V32"/>
-    <mergeCell ref="O33:V33"/>
-    <mergeCell ref="O34:V34"/>
-    <mergeCell ref="O35:V35"/>
-    <mergeCell ref="O36:V36"/>
-    <mergeCell ref="O37:V37"/>
-    <mergeCell ref="O38:V38"/>
-    <mergeCell ref="O39:V39"/>
-    <mergeCell ref="O40:V40"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="F44:K44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="O44:R44"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:K49"/>
-    <mergeCell ref="M49:N49"/>
-    <mergeCell ref="O49:R49"/>
+    <mergeCell ref="C4:M4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:O5"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="O7:S9"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="F1:H2"/>
+    <mergeCell ref="I1:U1"/>
+    <mergeCell ref="J2:U2"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="R3:S3"/>
   </mergeCells>
   <conditionalFormatting sqref="A10:F10 A40:N40 W10:W40 A11:D39">
     <cfRule type="expression" dxfId="839" priority="871" stopIfTrue="1">

</xml_diff>